<commit_message>
Befororethe big update of 02 stage
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/HZD_Focus/tables/env_cutoff_metrics.xlsx
+++ b/results/01_pollution_assessment/HZD_Focus/tables/env_cutoff_metrics.xlsx
@@ -488,31 +488,31 @@
         <v>0.05</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5493441386153743</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09868827723074869</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F2" t="n">
-        <v>1.218988114184364</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G2" t="n">
-        <v>0.302</v>
+        <v>0.17</v>
       </c>
       <c r="H2" t="n">
-        <v>140.3024337922869</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I2" t="n">
-        <v>255.3998922167808</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J2" t="n">
-        <v>6.499935558283235</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K2" t="n">
-        <v>1.954380260166737</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="3">
@@ -523,31 +523,31 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4089961524571829</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1134942286857743</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F3" t="n">
-        <v>1.384072723579188</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G3" t="n">
-        <v>0.119</v>
+        <v>0.164</v>
       </c>
       <c r="H3" t="n">
-        <v>139.8367242727358</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I3" t="n">
-        <v>341.9022976930696</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J3" t="n">
-        <v>4.308191149960391</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K3" t="n">
-        <v>1.974744694275297</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="4">
@@ -558,31 +558,31 @@
         <v>0.09</v>
       </c>
       <c r="C4" t="n">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3594128661761966</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1306317469534096</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F4" t="n">
-        <v>1.5709900685738</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G4" t="n">
-        <v>0.028</v>
+        <v>0.159</v>
       </c>
       <c r="H4" t="n">
-        <v>180.9038968423562</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I4" t="n">
-        <v>503.3317220026033</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J4" t="n">
-        <v>4.019653725918261</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K4" t="n">
-        <v>1.793822282115788</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="5">
@@ -593,31 +593,31 @@
         <v>0.11</v>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3141293014697661</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1336370123828625</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F5" t="n">
-        <v>1.740402889557896</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G5" t="n">
-        <v>0.007</v>
+        <v>0.148</v>
       </c>
       <c r="H5" t="n">
-        <v>176.7934989382114</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I5" t="n">
-        <v>562.8048644651101</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J5" t="n">
-        <v>3.110231745843306</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K5" t="n">
-        <v>1.460015560485308</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="6">
@@ -628,31 +628,31 @@
         <v>0.13</v>
       </c>
       <c r="C6" t="n">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2781603808501816</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1277771268606361</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F6" t="n">
-        <v>1.849676566178832</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G6" t="n">
-        <v>0.004</v>
+        <v>0.154</v>
       </c>
       <c r="H6" t="n">
-        <v>185.7045124075011</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I6" t="n">
-        <v>667.6166887602958</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J6" t="n">
-        <v>3.14247095110328</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K6" t="n">
-        <v>1.370665865789714</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="7">
@@ -663,31 +663,31 @@
         <v>0.15</v>
       </c>
       <c r="C7" t="n">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2872868375218746</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E7" t="n">
-        <v>0.160016629936495</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F7" t="n">
-        <v>2.257298412349547</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G7" t="n">
-        <v>0.002</v>
+        <v>0.151</v>
       </c>
       <c r="H7" t="n">
-        <v>239.9666015014136</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I7" t="n">
-        <v>835.2857498497199</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J7" t="n">
-        <v>4.376674967773068</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K7" t="n">
-        <v>1.311881922546723</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="8">
@@ -698,31 +698,31 @@
         <v>0.17</v>
       </c>
       <c r="C8" t="n">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2595810427990405</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1473963523140466</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F8" t="n">
-        <v>2.313872255446145</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001</v>
+        <v>0.175</v>
       </c>
       <c r="H8" t="n">
-        <v>241.6241974676451</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I8" t="n">
-        <v>930.8237414498062</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J8" t="n">
-        <v>3.779319586352292</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K8" t="n">
-        <v>1.102152159768521</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="9">
@@ -733,31 +733,31 @@
         <v>0.19</v>
       </c>
       <c r="C9" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1862357283293831</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E9" t="n">
-        <v>0.07916148205693363</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F9" t="n">
-        <v>1.739313932273759</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G9" t="n">
-        <v>0.007</v>
+        <v>0.135</v>
       </c>
       <c r="H9" t="n">
-        <v>187.828642887287</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I9" t="n">
-        <v>1008.553216787096</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J9" t="n">
-        <v>2.234309019106088</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K9" t="n">
-        <v>1.081610666460168</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="10">
@@ -768,31 +768,31 @@
         <v>0.21</v>
       </c>
       <c r="C10" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1452929879530765</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E10" t="n">
-        <v>0.04354215318558563</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F10" t="n">
-        <v>1.427929198665377</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G10" t="n">
-        <v>0.051</v>
+        <v>0.148</v>
       </c>
       <c r="H10" t="n">
-        <v>158.4947034060169</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I10" t="n">
-        <v>1090.86271566804</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J10" t="n">
-        <v>1.855338287430084</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K10" t="n">
-        <v>1.127674926690246</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="11">
@@ -803,31 +803,31 @@
         <v>0.23</v>
       </c>
       <c r="C11" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1433433030564309</v>
+        <v>0.1148679210081479</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0522096118922214</v>
+        <v>0.02809026620502508</v>
       </c>
       <c r="F11" t="n">
-        <v>1.572890346317121</v>
+        <v>1.323703910514234</v>
       </c>
       <c r="G11" t="n">
-        <v>0.023</v>
+        <v>0.164</v>
       </c>
       <c r="H11" t="n">
-        <v>169.4997121280336</v>
+        <v>2.339713099696875</v>
       </c>
       <c r="I11" t="n">
-        <v>1182.473882726879</v>
+        <v>20.36872504666393</v>
       </c>
       <c r="J11" t="n">
-        <v>1.747092713206695</v>
+        <v>0.03012478423244144</v>
       </c>
       <c r="K11" t="n">
-        <v>1.132558506324056</v>
+        <v>1.114138135674124</v>
       </c>
     </row>
     <row r="12">
@@ -841,28 +841,28 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1328967290176022</v>
+        <v>0.1009661331288063</v>
       </c>
       <c r="E12" t="n">
-        <v>0.04952141450006387</v>
+        <v>0.01452056900657606</v>
       </c>
       <c r="F12" t="n">
-        <v>1.5939577534025</v>
+        <v>1.167973558319831</v>
       </c>
       <c r="G12" t="n">
-        <v>0.018</v>
+        <v>0.288</v>
       </c>
       <c r="H12" t="n">
-        <v>165.5323820946634</v>
+        <v>2.083308709738726</v>
       </c>
       <c r="I12" t="n">
-        <v>1245.571530001605</v>
+        <v>20.63373772154839</v>
       </c>
       <c r="J12" t="n">
-        <v>1.513430057122149</v>
+        <v>0.02346348358492378</v>
       </c>
       <c r="K12" t="n">
-        <v>1.11347015706863</v>
+        <v>1.214322660478865</v>
       </c>
     </row>
     <row r="13">
@@ -876,28 +876,28 @@
         <v>62</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1225195504250746</v>
+        <v>0.1047642240513707</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0441730817130277</v>
+        <v>0.0248324583416718</v>
       </c>
       <c r="F13" t="n">
-        <v>1.563817137379612</v>
+        <v>1.310670709212902</v>
       </c>
       <c r="G13" t="n">
-        <v>0.018</v>
+        <v>0.171</v>
       </c>
       <c r="H13" t="n">
-        <v>159.7871290781582</v>
+        <v>2.354666361301749</v>
       </c>
       <c r="I13" t="n">
-        <v>1304.176586706251</v>
+        <v>22.47586313575088</v>
       </c>
       <c r="J13" t="n">
-        <v>1.255679551953282</v>
+        <v>0.02550671852782241</v>
       </c>
       <c r="K13" t="n">
-        <v>1.109627119822215</v>
+        <v>1.159530828463135</v>
       </c>
     </row>
     <row r="14">
@@ -911,28 +911,28 @@
         <v>67</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1286395183075753</v>
+        <v>0.09894930964850776</v>
       </c>
       <c r="E14" t="n">
-        <v>0.05721652800491739</v>
+        <v>0.02509269568527062</v>
       </c>
       <c r="F14" t="n">
-        <v>1.80109398615852</v>
+        <v>1.339748796198007</v>
       </c>
       <c r="G14" t="n">
-        <v>0.01</v>
+        <v>0.159</v>
       </c>
       <c r="H14" t="n">
-        <v>179.2966913428212</v>
+        <v>2.421712425162892</v>
       </c>
       <c r="I14" t="n">
-        <v>1393.791687824307</v>
+        <v>24.47427307745156</v>
       </c>
       <c r="J14" t="n">
-        <v>1.229166009882097</v>
+        <v>0.02395746937069712</v>
       </c>
       <c r="K14" t="n">
-        <v>1.186305791510718</v>
+        <v>1.183658605454276</v>
       </c>
     </row>
     <row r="15">
@@ -946,28 +946,28 @@
         <v>72</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1296514503413271</v>
+        <v>0.09835348811129903</v>
       </c>
       <c r="E15" t="n">
-        <v>0.06371595415506404</v>
+        <v>0.03004693418033699</v>
       </c>
       <c r="F15" t="n">
-        <v>1.966337676068608</v>
+        <v>1.439883619523617</v>
       </c>
       <c r="G15" t="n">
-        <v>0.002</v>
+        <v>0.098</v>
       </c>
       <c r="H15" t="n">
-        <v>198.5194929146411</v>
+        <v>2.50680952000912</v>
       </c>
       <c r="I15" t="n">
-        <v>1531.178343103825</v>
+        <v>25.48775410153586</v>
       </c>
       <c r="J15" t="n">
-        <v>1.174112804607233</v>
+        <v>0.02191537611357883</v>
       </c>
       <c r="K15" t="n">
-        <v>1.240960547568766</v>
+        <v>1.201657520819642</v>
       </c>
     </row>
     <row r="16">
@@ -981,28 +981,28 @@
         <v>76</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1271688652474025</v>
+        <v>0.0944904025343976</v>
       </c>
       <c r="E16" t="n">
-        <v>0.06482378419364554</v>
+        <v>0.02981114557256881</v>
       </c>
       <c r="F16" t="n">
-        <v>2.039757798016996</v>
+        <v>1.460907359992744</v>
       </c>
       <c r="G16" t="n">
-        <v>0.003</v>
+        <v>0.102</v>
       </c>
       <c r="H16" t="n">
-        <v>200.6425805605473</v>
+        <v>2.607046432723598</v>
       </c>
       <c r="I16" t="n">
-        <v>1577.764967629493</v>
+        <v>27.59059505302189</v>
       </c>
       <c r="J16" t="n">
-        <v>1.163641762731222</v>
+        <v>0.02170330874664016</v>
       </c>
       <c r="K16" t="n">
-        <v>1.252939231560085</v>
+        <v>1.221986025880401</v>
       </c>
     </row>
     <row r="17">
@@ -1016,28 +1016,28 @@
         <v>81</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1387446418274837</v>
+        <v>0.09004682363281571</v>
       </c>
       <c r="E17" t="n">
-        <v>0.08132761794931598</v>
+        <v>0.02938327854167011</v>
       </c>
       <c r="F17" t="n">
-        <v>2.416437363975599</v>
+        <v>1.484364678943876</v>
       </c>
       <c r="G17" t="n">
-        <v>0.001</v>
+        <v>0.081</v>
       </c>
       <c r="H17" t="n">
-        <v>244.196086519077</v>
+        <v>2.675965807533299</v>
       </c>
       <c r="I17" t="n">
-        <v>1760.039762996488</v>
+        <v>29.71749251750506</v>
       </c>
       <c r="J17" t="n">
-        <v>1.584616993505296</v>
+        <v>0.01943423086047135</v>
       </c>
       <c r="K17" t="n">
-        <v>1.234073163047965</v>
+        <v>1.231331948343868</v>
       </c>
     </row>
     <row r="18">
@@ -1051,28 +1051,28 @@
         <v>86</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1392333421490901</v>
+        <v>0.09407651429428682</v>
       </c>
       <c r="E18" t="n">
-        <v>0.08543542603340826</v>
+        <v>0.03745629643767967</v>
       </c>
       <c r="F18" t="n">
-        <v>2.58808058382217</v>
+        <v>1.661535717374654</v>
       </c>
       <c r="G18" t="n">
-        <v>0.001</v>
+        <v>0.036</v>
       </c>
       <c r="H18" t="n">
-        <v>258.7011553434654</v>
+        <v>2.966116972510829</v>
       </c>
       <c r="I18" t="n">
-        <v>1858.040260690217</v>
+        <v>31.52877202946026</v>
       </c>
       <c r="J18" t="n">
-        <v>1.752502622324773</v>
+        <v>0.01984112686961536</v>
       </c>
       <c r="K18" t="n">
-        <v>1.244794341061955</v>
+        <v>1.256411632303104</v>
       </c>
     </row>
     <row r="19">
@@ -1086,28 +1086,28 @@
         <v>90</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1377253516368927</v>
+        <v>0.1097732365698765</v>
       </c>
       <c r="E19" t="n">
-        <v>0.08639947971051731</v>
+        <v>0.05678354827046439</v>
       </c>
       <c r="F19" t="n">
-        <v>2.683351426244709</v>
+        <v>2.071596193387955</v>
       </c>
       <c r="G19" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="H19" t="n">
-        <v>260.2651154272517</v>
+        <v>3.704354325052696</v>
       </c>
       <c r="I19" t="n">
-        <v>1889.740068432935</v>
+        <v>33.74551430570855</v>
       </c>
       <c r="J19" t="n">
-        <v>1.754674351185182</v>
+        <v>0.0248215105929011</v>
       </c>
       <c r="K19" t="n">
-        <v>1.239159144586637</v>
+        <v>1.246992608756951</v>
       </c>
     </row>
     <row r="20">
@@ -1121,28 +1121,28 @@
         <v>95</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1549524857014103</v>
+        <v>0.1192000012167057</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1074779062464334</v>
+        <v>0.06971685521764426</v>
       </c>
       <c r="F20" t="n">
-        <v>3.263904335337214</v>
+        <v>2.408901027007591</v>
       </c>
       <c r="G20" t="n">
         <v>0.001</v>
       </c>
       <c r="H20" t="n">
-        <v>317.4968344975641</v>
+        <v>4.19145057321373</v>
       </c>
       <c r="I20" t="n">
-        <v>2048.994780950935</v>
+        <v>35.16317559085985</v>
       </c>
       <c r="J20" t="n">
-        <v>2.215035000726104</v>
+        <v>0.0261948013040817</v>
       </c>
       <c r="K20" t="n">
-        <v>1.230991182334984</v>
+        <v>1.25011431627727</v>
       </c>
     </row>
     <row r="21">
@@ -1156,28 +1156,28 @@
         <v>100</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1502377113957074</v>
+        <v>0.1201146741430924</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1050375896614366</v>
+        <v>0.07331226319325701</v>
       </c>
       <c r="F21" t="n">
-        <v>3.323834220601151</v>
+        <v>2.566420654522169</v>
       </c>
       <c r="G21" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="H21" t="n">
-        <v>324.4132941147163</v>
+        <v>4.356464560582069</v>
       </c>
       <c r="I21" t="n">
-        <v>2159.333306537479</v>
+        <v>36.26921183162201</v>
       </c>
       <c r="J21" t="n">
-        <v>2.122403526844773</v>
+        <v>0.02507788370311485</v>
       </c>
       <c r="K21" t="n">
-        <v>1.291753165940297</v>
+        <v>1.290731747181407</v>
       </c>
     </row>
     <row r="22">
@@ -1188,31 +1188,31 @@
         <v>0.45</v>
       </c>
       <c r="C22" t="n">
-        <v>104</v>
+        <v>233</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1485358544376552</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1050938061946785</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F22" t="n">
-        <v>3.4191724480134</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G22" t="n">
         <v>0.001</v>
       </c>
       <c r="H22" t="n">
-        <v>329.2800400568107</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I22" t="n">
-        <v>2216.838764643315</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J22" t="n">
-        <v>2.021022108763582</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K22" t="n">
-        <v>1.277207209213268</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="23">
@@ -1223,31 +1223,31 @@
         <v>0.47</v>
       </c>
       <c r="C23" t="n">
-        <v>109</v>
+        <v>233</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1404782697604895</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E23" t="n">
-        <v>0.09875391392362021</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F23" t="n">
-        <v>3.366816981182892</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G23" t="n">
         <v>0.001</v>
       </c>
       <c r="H23" t="n">
-        <v>327.7781453439064</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I23" t="n">
-        <v>2333.301413113619</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J23" t="n">
-        <v>1.965314818274389</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K23" t="n">
-        <v>1.220959462116517</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="24">
@@ -1258,31 +1258,31 @@
         <v>0.49</v>
       </c>
       <c r="C24" t="n">
-        <v>114</v>
+        <v>233</v>
       </c>
       <c r="D24" t="n">
-        <v>0.1343963550134016</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0943221121899479</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F24" t="n">
-        <v>3.353684200734182</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G24" t="n">
         <v>0.001</v>
       </c>
       <c r="H24" t="n">
-        <v>334.9076511341209</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I24" t="n">
-        <v>2491.93998677066</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J24" t="n">
-        <v>2.003906862937082</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K24" t="n">
-        <v>1.21022092471995</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="25">
@@ -1293,31 +1293,31 @@
         <v>0.51</v>
       </c>
       <c r="C25" t="n">
-        <v>118</v>
+        <v>233</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1503535450313161</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E25" t="n">
-        <v>0.112422899720214</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F25" t="n">
-        <v>3.96390685679447</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G25" t="n">
         <v>0.001</v>
       </c>
       <c r="H25" t="n">
-        <v>403.9225978641679</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I25" t="n">
-        <v>2686.485362084663</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J25" t="n">
-        <v>2.573002842009365</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K25" t="n">
-        <v>1.237677418015282</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="26">
@@ -1328,31 +1328,31 @@
         <v>0.53</v>
       </c>
       <c r="C26" t="n">
-        <v>123</v>
+        <v>233</v>
       </c>
       <c r="D26" t="n">
-        <v>0.1540535230379662</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1179019641934347</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F26" t="n">
-        <v>4.261324489504545</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G26" t="n">
         <v>0.001</v>
       </c>
       <c r="H26" t="n">
-        <v>433.8342934500299</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I26" t="n">
-        <v>2816.127050486943</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J26" t="n">
-        <v>2.688380165329499</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K26" t="n">
-        <v>1.215390296200202</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="27">
@@ -1363,31 +1363,31 @@
         <v>0.55</v>
       </c>
       <c r="C27" t="n">
-        <v>128</v>
+        <v>233</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1561751904593513</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1215922064617837</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F27" t="n">
-        <v>4.515954738617582</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G27" t="n">
         <v>0.001</v>
       </c>
       <c r="H27" t="n">
-        <v>453.4092216221998</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I27" t="n">
-        <v>2903.209019874456</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J27" t="n">
-        <v>2.649429463012936</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K27" t="n">
-        <v>1.244228131755367</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="28">
@@ -1398,31 +1398,31 @@
         <v>0.57</v>
       </c>
       <c r="C28" t="n">
-        <v>132</v>
+        <v>233</v>
       </c>
       <c r="D28" t="n">
-        <v>0.160109122369278</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1267801192886937</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F28" t="n">
-        <v>4.803897733819392</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G28" t="n">
         <v>0.001</v>
       </c>
       <c r="H28" t="n">
-        <v>480.0456283163218</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I28" t="n">
-        <v>2998.240332672223</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J28" t="n">
-        <v>2.761113888670642</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K28" t="n">
-        <v>1.248807337371973</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="29">
@@ -1433,31 +1433,31 @@
         <v>0.59</v>
       </c>
       <c r="C29" t="n">
-        <v>137</v>
+        <v>233</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1699095447834601</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1382267029813021</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F29" t="n">
-        <v>5.362825274464079</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G29" t="n">
         <v>0.001</v>
       </c>
       <c r="H29" t="n">
-        <v>544.3056293713004</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I29" t="n">
-        <v>3203.502369834411</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J29" t="n">
-        <v>3.114381686215466</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K29" t="n">
-        <v>1.289873874467393</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="30">
@@ -1468,31 +1468,31 @@
         <v>0.61</v>
       </c>
       <c r="C30" t="n">
-        <v>142</v>
+        <v>233</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1671504790493253</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E30" t="n">
-        <v>0.1365310113673152</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F30" t="n">
-        <v>5.458960971667431</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G30" t="n">
         <v>0.001</v>
       </c>
       <c r="H30" t="n">
-        <v>564.3583863574108</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I30" t="n">
-        <v>3376.349200835202</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J30" t="n">
-        <v>3.120267912726051</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K30" t="n">
-        <v>1.251646565976789</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="31">
@@ -1503,31 +1503,31 @@
         <v>0.63</v>
       </c>
       <c r="C31" t="n">
-        <v>146</v>
+        <v>233</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1674816138281158</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E31" t="n">
-        <v>0.1377488143219771</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F31" t="n">
-        <v>5.632890834700483</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G31" t="n">
         <v>0.001</v>
       </c>
       <c r="H31" t="n">
-        <v>582.0087257212795</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I31" t="n">
-        <v>3475.060410622669</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J31" t="n">
-        <v>3.178264790622704</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K31" t="n">
-        <v>1.254236550930427</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="32">
@@ -1538,31 +1538,31 @@
         <v>0.65</v>
       </c>
       <c r="C32" t="n">
-        <v>151</v>
+        <v>233</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1735047216247679</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E32" t="n">
-        <v>0.1450048844394149</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F32" t="n">
-        <v>6.087919748325392</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G32" t="n">
         <v>0.001</v>
       </c>
       <c r="H32" t="n">
-        <v>634.5975457590848</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I32" t="n">
-        <v>3657.523206379969</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J32" t="n">
-        <v>3.37076048810545</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K32" t="n">
-        <v>1.255000143517022</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="33">
@@ -1573,31 +1573,31 @@
         <v>0.67</v>
       </c>
       <c r="C33" t="n">
-        <v>156</v>
+        <v>233</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1792540658979996</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E33" t="n">
-        <v>0.1518958680945994</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F33" t="n">
-        <v>6.552115281355348</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G33" t="n">
         <v>0.001</v>
       </c>
       <c r="H33" t="n">
-        <v>685.9547609513362</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I33" t="n">
-        <v>3826.718002266476</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J33" t="n">
-        <v>3.54259975888812</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K33" t="n">
-        <v>1.267108691557905</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="34">
@@ -1608,31 +1608,31 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="C34" t="n">
-        <v>160</v>
+        <v>233</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1821415739611562</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E34" t="n">
-        <v>0.155587728959895</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F34" t="n">
-        <v>6.859329560464992</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G34" t="n">
         <v>0.001</v>
       </c>
       <c r="H34" t="n">
-        <v>736.4838801865226</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I34" t="n">
-        <v>4043.469396742922</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J34" t="n">
-        <v>3.738009994350619</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K34" t="n">
-        <v>1.280993126056221</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="35">
@@ -1643,31 +1643,31 @@
         <v>0.71</v>
       </c>
       <c r="C35" t="n">
-        <v>165</v>
+        <v>233</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1815534738219688</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E35" t="n">
-        <v>0.1558161616780056</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F35" t="n">
-        <v>7.0540961234195</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G35" t="n">
         <v>0.001</v>
       </c>
       <c r="H35" t="n">
-        <v>754.9835215996958</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I35" t="n">
-        <v>4158.463650990408</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J35" t="n">
-        <v>3.756665631614881</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K35" t="n">
-        <v>1.288731883811476</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="36">
@@ -1678,31 +1678,31 @@
         <v>0.73</v>
       </c>
       <c r="C36" t="n">
-        <v>170</v>
+        <v>233</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1828586921459113</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E36" t="n">
-        <v>0.1579458473942622</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F36" t="n">
-        <v>7.33993624448719</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G36" t="n">
         <v>0.001</v>
       </c>
       <c r="H36" t="n">
-        <v>783.1212998881103</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I36" t="n">
-        <v>4282.658323199764</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J36" t="n">
-        <v>3.832909971498491</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K36" t="n">
-        <v>1.278592205447013</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="37">
@@ -1713,31 +1713,31 @@
         <v>0.75</v>
       </c>
       <c r="C37" t="n">
-        <v>174</v>
+        <v>233</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1832939543894962</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1589872268415646</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F37" t="n">
-        <v>7.540873366357098</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G37" t="n">
         <v>0.001</v>
       </c>
       <c r="H37" t="n">
-        <v>797.3485622751706</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I37" t="n">
-        <v>4350.10835426039</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J37" t="n">
-        <v>3.815494179467918</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K37" t="n">
-        <v>1.253923317457474</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="38">
@@ -1748,31 +1748,31 @@
         <v>0.77</v>
       </c>
       <c r="C38" t="n">
-        <v>179</v>
+        <v>233</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1792910797552772</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1555711687655452</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F38" t="n">
-        <v>7.558674222381804</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G38" t="n">
         <v>0.001</v>
       </c>
       <c r="H38" t="n">
-        <v>802.0872979642154</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I38" t="n">
-        <v>4473.659810956697</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J38" t="n">
-        <v>3.742525729603451</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K38" t="n">
-        <v>1.233805270660643</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="39">
@@ -1783,31 +1783,31 @@
         <v>0.79</v>
       </c>
       <c r="C39" t="n">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1809411008154943</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1579338283664914</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F39" t="n">
-        <v>7.86451767442496</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G39" t="n">
         <v>0.001</v>
       </c>
       <c r="H39" t="n">
-        <v>838.3532757570998</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I39" t="n">
-        <v>4633.293773380814</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J39" t="n">
-        <v>3.847369118827479</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K39" t="n">
-        <v>1.261660173417972</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="40">
@@ -1818,31 +1818,31 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="C40" t="n">
-        <v>188</v>
+        <v>233</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1785163605935729</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E40" t="n">
-        <v>0.155948128741748</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F40" t="n">
-        <v>7.910072962988355</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G40" t="n">
         <v>0.001</v>
       </c>
       <c r="H40" t="n">
-        <v>840.7778813350751</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I40" t="n">
-        <v>4709.808549420683</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J40" t="n">
-        <v>3.794906976292337</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K40" t="n">
-        <v>1.262686227746374</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="41">
@@ -1853,31 +1853,31 @@
         <v>0.83</v>
       </c>
       <c r="C41" t="n">
-        <v>193</v>
+        <v>233</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1784833765359438</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1565176914165839</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F41" t="n">
-        <v>8.125554726204959</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G41" t="n">
         <v>0.001</v>
       </c>
       <c r="H41" t="n">
-        <v>874.0839910630057</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I41" t="n">
-        <v>4897.285159141857</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J41" t="n">
-        <v>3.903076434031391</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K41" t="n">
-        <v>1.240736105451826</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="42">
@@ -1888,31 +1888,31 @@
         <v>0.85</v>
       </c>
       <c r="C42" t="n">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1897781161581535</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1686785879331054</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F42" t="n">
-        <v>8.994424620966663</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G42" t="n">
         <v>0.001</v>
       </c>
       <c r="H42" t="n">
-        <v>960.4790539823404</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I42" t="n">
-        <v>5061.063274450018</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J42" t="n">
-        <v>4.248461821288234</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K42" t="n">
-        <v>1.226518146656127</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="43">
@@ -1923,31 +1923,31 @@
         <v>0.87</v>
       </c>
       <c r="C43" t="n">
-        <v>202</v>
+        <v>233</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1827941031391985</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1619470139335658</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F43" t="n">
-        <v>8.768327383077022</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G43" t="n">
         <v>0.001</v>
       </c>
       <c r="H43" t="n">
-        <v>942.1072842244968</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I43" t="n">
-        <v>5153.926018647757</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J43" t="n">
-        <v>4.078807811535828</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K43" t="n">
-        <v>1.22510859832298</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="44">
@@ -1958,31 +1958,31 @@
         <v>0.89</v>
       </c>
       <c r="C44" t="n">
-        <v>207</v>
+        <v>233</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1876174667839904</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E44" t="n">
-        <v>0.167408946057224</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F44" t="n">
-        <v>9.284077212810981</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G44" t="n">
         <v>0.001</v>
       </c>
       <c r="H44" t="n">
-        <v>1001.54829058189</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I44" t="n">
-        <v>5338.246527627422</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J44" t="n">
-        <v>4.275839716927726</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K44" t="n">
-        <v>1.216195208342588</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="45">
@@ -1993,31 +1993,31 @@
         <v>0.91</v>
       </c>
       <c r="C45" t="n">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1897183966904346</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1700513674838918</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F45" t="n">
-        <v>9.646520310618083</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G45" t="n">
         <v>0.001</v>
       </c>
       <c r="H45" t="n">
-        <v>1035.405991049978</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I45" t="n">
-        <v>5457.594039967878</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J45" t="n">
-        <v>4.289326198092065</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K45" t="n">
-        <v>1.218860721001413</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="46">
@@ -2028,31 +2028,31 @@
         <v>0.93</v>
       </c>
       <c r="C46" t="n">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1960073387177583</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1768646563062765</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F46" t="n">
-        <v>10.23928279770193</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G46" t="n">
         <v>0.001</v>
       </c>
       <c r="H46" t="n">
-        <v>1096.418464023794</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I46" t="n">
-        <v>5593.762311127477</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J46" t="n">
-        <v>4.491113780404402</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K46" t="n">
-        <v>1.210964632501354</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="47">
@@ -2063,31 +2063,31 @@
         <v>0.95</v>
       </c>
       <c r="C47" t="n">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1956279833743561</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1769216574063178</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F47" t="n">
-        <v>10.45785172933517</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G47" t="n">
         <v>0.001</v>
       </c>
       <c r="H47" t="n">
-        <v>1125.911386126806</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I47" t="n">
-        <v>5755.369792736903</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J47" t="n">
-        <v>4.532469062133008</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K47" t="n">
-        <v>1.221252557534644</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="48">
@@ -2098,31 +2098,31 @@
         <v>0.97</v>
       </c>
       <c r="C48" t="n">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1939955310668408</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1756772476819962</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F48" t="n">
-        <v>10.59026803938088</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G48" t="n">
         <v>0.001</v>
       </c>
       <c r="H48" t="n">
-        <v>1146.675325992493</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I48" t="n">
-        <v>5910.833717078816</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J48" t="n">
-        <v>4.478926482981763</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K48" t="n">
-        <v>1.221978297960755</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
     <row r="49">
@@ -2133,31 +2133,31 @@
         <v>0.99</v>
       </c>
       <c r="C49" t="n">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D49" t="n">
-        <v>0.1822022305391026</v>
+        <v>0.1811449267518876</v>
       </c>
       <c r="E49" t="n">
-        <v>0.1639478160422075</v>
+        <v>0.1631084713939998</v>
       </c>
       <c r="F49" t="n">
-        <v>9.981269493474803</v>
+        <v>10.04326643775198</v>
       </c>
       <c r="G49" t="n">
         <v>0.001</v>
       </c>
       <c r="H49" t="n">
-        <v>1095.089815496517</v>
+        <v>19.18414947938523</v>
       </c>
       <c r="I49" t="n">
-        <v>6010.298623986928</v>
+        <v>105.9049779829692</v>
       </c>
       <c r="J49" t="n">
-        <v>4.177739388609544</v>
+        <v>0.07330599712226725</v>
       </c>
       <c r="K49" t="n">
-        <v>1.21207697077835</v>
+        <v>1.221558912811017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Before ch2 results update.
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/HZD_Focus/tables/env_cutoff_metrics.xlsx
+++ b/results/01_pollution_assessment/HZD_Focus/tables/env_cutoff_metrics.xlsx
@@ -491,25 +491,25 @@
         <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F2" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G2" t="n">
-        <v>0.17</v>
+        <v>0.013</v>
       </c>
       <c r="H2" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I2" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J2" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K2" t="n">
         <v>1.114138135674124</v>
@@ -526,25 +526,25 @@
         <v>57</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F3" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G3" t="n">
-        <v>0.164</v>
+        <v>0.013</v>
       </c>
       <c r="H3" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I3" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J3" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K3" t="n">
         <v>1.114138135674124</v>
@@ -561,25 +561,25 @@
         <v>57</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F4" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G4" t="n">
-        <v>0.159</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I4" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J4" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K4" t="n">
         <v>1.114138135674124</v>
@@ -596,25 +596,25 @@
         <v>57</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F5" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G5" t="n">
-        <v>0.148</v>
+        <v>0.012</v>
       </c>
       <c r="H5" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I5" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J5" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K5" t="n">
         <v>1.114138135674124</v>
@@ -631,25 +631,25 @@
         <v>57</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E6" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F6" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G6" t="n">
-        <v>0.154</v>
+        <v>0.011</v>
       </c>
       <c r="H6" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I6" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J6" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K6" t="n">
         <v>1.114138135674124</v>
@@ -666,25 +666,25 @@
         <v>57</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E7" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F7" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G7" t="n">
-        <v>0.151</v>
+        <v>0.014</v>
       </c>
       <c r="H7" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I7" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J7" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K7" t="n">
         <v>1.114138135674124</v>
@@ -701,25 +701,25 @@
         <v>57</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E8" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F8" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G8" t="n">
-        <v>0.175</v>
+        <v>0.016</v>
       </c>
       <c r="H8" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I8" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J8" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K8" t="n">
         <v>1.114138135674124</v>
@@ -736,25 +736,25 @@
         <v>57</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E9" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F9" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G9" t="n">
-        <v>0.135</v>
+        <v>0.007</v>
       </c>
       <c r="H9" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I9" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J9" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K9" t="n">
         <v>1.114138135674124</v>
@@ -771,25 +771,25 @@
         <v>57</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E10" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F10" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G10" t="n">
-        <v>0.148</v>
+        <v>0.011</v>
       </c>
       <c r="H10" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I10" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J10" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K10" t="n">
         <v>1.114138135674124</v>
@@ -806,25 +806,25 @@
         <v>57</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1148679210081479</v>
+        <v>0.140841332851933</v>
       </c>
       <c r="E11" t="n">
-        <v>0.02809026620502508</v>
+        <v>0.05661009097467129</v>
       </c>
       <c r="F11" t="n">
-        <v>1.323703910514234</v>
+        <v>1.672079500586748</v>
       </c>
       <c r="G11" t="n">
-        <v>0.164</v>
+        <v>0.015</v>
       </c>
       <c r="H11" t="n">
-        <v>2.339713099696875</v>
+        <v>168.1302198445361</v>
       </c>
       <c r="I11" t="n">
-        <v>20.36872504666393</v>
+        <v>1193.756239308613</v>
       </c>
       <c r="J11" t="n">
-        <v>0.03012478423244144</v>
+        <v>1.675921196794977</v>
       </c>
       <c r="K11" t="n">
         <v>1.114138135674124</v>
@@ -841,25 +841,25 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1009661331288063</v>
+        <v>0.148950191688079</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01452056900657606</v>
+        <v>0.06711847935039417</v>
       </c>
       <c r="F12" t="n">
-        <v>1.167973558319831</v>
+        <v>1.820201330670252</v>
       </c>
       <c r="G12" t="n">
-        <v>0.288</v>
+        <v>0.006</v>
       </c>
       <c r="H12" t="n">
-        <v>2.083308709738726</v>
+        <v>181.9385729227985</v>
       </c>
       <c r="I12" t="n">
-        <v>20.63373772154839</v>
+        <v>1221.472566506</v>
       </c>
       <c r="J12" t="n">
-        <v>0.02346348358492378</v>
+        <v>1.713906237294484</v>
       </c>
       <c r="K12" t="n">
         <v>1.214322660478865</v>
@@ -876,25 +876,25 @@
         <v>62</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1047642240513707</v>
+        <v>0.1546736990028364</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0248324583416718</v>
+        <v>0.07919813641380391</v>
       </c>
       <c r="F13" t="n">
-        <v>1.310670709212902</v>
+        <v>2.04932157770113</v>
       </c>
       <c r="G13" t="n">
-        <v>0.171</v>
+        <v>0.003</v>
       </c>
       <c r="H13" t="n">
-        <v>2.354666361301749</v>
+        <v>204.6601133805163</v>
       </c>
       <c r="I13" t="n">
-        <v>22.47586313575088</v>
+        <v>1323.17333004859</v>
       </c>
       <c r="J13" t="n">
-        <v>0.02550671852782241</v>
+        <v>2.080661386350577</v>
       </c>
       <c r="K13" t="n">
         <v>1.159530828463135</v>
@@ -911,25 +911,25 @@
         <v>67</v>
       </c>
       <c r="D14" t="n">
-        <v>0.09894930964850776</v>
+        <v>0.1461792616319332</v>
       </c>
       <c r="E14" t="n">
-        <v>0.02509269568527062</v>
+        <v>0.07619395520832117</v>
       </c>
       <c r="F14" t="n">
-        <v>1.339748796198007</v>
+        <v>2.088713604354735</v>
       </c>
       <c r="G14" t="n">
-        <v>0.159</v>
+        <v>0.001</v>
       </c>
       <c r="H14" t="n">
-        <v>2.421712425162892</v>
+        <v>210.7389194016748</v>
       </c>
       <c r="I14" t="n">
-        <v>24.47427307745156</v>
+        <v>1441.647173812502</v>
       </c>
       <c r="J14" t="n">
-        <v>0.02395746937069712</v>
+        <v>1.954129417978096</v>
       </c>
       <c r="K14" t="n">
         <v>1.183658605454276</v>
@@ -946,25 +946,25 @@
         <v>72</v>
       </c>
       <c r="D15" t="n">
-        <v>0.09835348811129903</v>
+        <v>0.1460319418268244</v>
       </c>
       <c r="E15" t="n">
-        <v>0.03004693418033699</v>
+        <v>0.08133739196522016</v>
       </c>
       <c r="F15" t="n">
-        <v>1.439883619523617</v>
+        <v>2.257252614620839</v>
       </c>
       <c r="G15" t="n">
-        <v>0.098</v>
+        <v>0.001</v>
       </c>
       <c r="H15" t="n">
-        <v>2.50680952000912</v>
+        <v>225.6519268868709</v>
       </c>
       <c r="I15" t="n">
-        <v>25.48775410153586</v>
+        <v>1545.223079718175</v>
       </c>
       <c r="J15" t="n">
-        <v>0.02191537611357883</v>
+        <v>1.762650600415906</v>
       </c>
       <c r="K15" t="n">
         <v>1.201657520819642</v>
@@ -981,25 +981,25 @@
         <v>76</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0944904025343976</v>
+        <v>0.1432770352249143</v>
       </c>
       <c r="E16" t="n">
-        <v>0.02981114557256881</v>
+        <v>0.08208253774097962</v>
       </c>
       <c r="F16" t="n">
-        <v>1.460907359992744</v>
+        <v>2.341338537219439</v>
       </c>
       <c r="G16" t="n">
-        <v>0.102</v>
+        <v>0.002</v>
       </c>
       <c r="H16" t="n">
-        <v>2.607046432723598</v>
+        <v>233.5826209987058</v>
       </c>
       <c r="I16" t="n">
-        <v>27.59059505302189</v>
+        <v>1630.286532883871</v>
       </c>
       <c r="J16" t="n">
-        <v>0.02170330874664016</v>
+        <v>1.716906825195904</v>
       </c>
       <c r="K16" t="n">
         <v>1.221986025880401</v>
@@ -1016,25 +1016,25 @@
         <v>81</v>
       </c>
       <c r="D17" t="n">
-        <v>0.09004682363281571</v>
+        <v>0.1310505550900521</v>
       </c>
       <c r="E17" t="n">
-        <v>0.02938327854167011</v>
+        <v>0.07312059209605559</v>
       </c>
       <c r="F17" t="n">
-        <v>1.484364678943876</v>
+        <v>2.262224042912531</v>
       </c>
       <c r="G17" t="n">
-        <v>0.081</v>
+        <v>0.001</v>
       </c>
       <c r="H17" t="n">
-        <v>2.675965807533299</v>
+        <v>225.0286644849758</v>
       </c>
       <c r="I17" t="n">
-        <v>29.71749251750506</v>
+        <v>1717.113402002351</v>
       </c>
       <c r="J17" t="n">
-        <v>0.01943423086047135</v>
+        <v>1.584468106419561</v>
       </c>
       <c r="K17" t="n">
         <v>1.231331948343868</v>
@@ -1051,25 +1051,25 @@
         <v>86</v>
       </c>
       <c r="D18" t="n">
-        <v>0.09407651429428682</v>
+        <v>0.1291550864205802</v>
       </c>
       <c r="E18" t="n">
-        <v>0.03745629643767967</v>
+        <v>0.0747272793218664</v>
       </c>
       <c r="F18" t="n">
-        <v>1.661535717374654</v>
+        <v>2.372961420002395</v>
       </c>
       <c r="G18" t="n">
-        <v>0.036</v>
+        <v>0.001</v>
       </c>
       <c r="H18" t="n">
-        <v>2.966116972510829</v>
+        <v>234.2249594121778</v>
       </c>
       <c r="I18" t="n">
-        <v>31.52877202946026</v>
+        <v>1813.517112670642</v>
       </c>
       <c r="J18" t="n">
-        <v>0.01984112686961536</v>
+        <v>1.568931275908667</v>
       </c>
       <c r="K18" t="n">
         <v>1.256411632303104</v>
@@ -1086,25 +1086,25 @@
         <v>90</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1097732365698765</v>
+        <v>0.150871919038706</v>
       </c>
       <c r="E19" t="n">
-        <v>0.05678354827046439</v>
+        <v>0.100328580886248</v>
       </c>
       <c r="F19" t="n">
-        <v>2.071596193387955</v>
+        <v>2.98500108132191</v>
       </c>
       <c r="G19" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="H19" t="n">
-        <v>3.704354325052696</v>
+        <v>292.4687654977014</v>
       </c>
       <c r="I19" t="n">
-        <v>33.74551430570855</v>
+        <v>1938.523532816395</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0248215105929011</v>
+        <v>2.092152607183344</v>
       </c>
       <c r="K19" t="n">
         <v>1.246992608756951</v>
@@ -1121,25 +1121,25 @@
         <v>95</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1192000012167057</v>
+        <v>0.1528531334189628</v>
       </c>
       <c r="E20" t="n">
-        <v>0.06971685521764426</v>
+        <v>0.1052606128245226</v>
       </c>
       <c r="F20" t="n">
-        <v>2.408901027007591</v>
+        <v>3.21170493829274</v>
       </c>
       <c r="G20" t="n">
         <v>0.001</v>
       </c>
       <c r="H20" t="n">
-        <v>4.19145057321373</v>
+        <v>314.2636850384355</v>
       </c>
       <c r="I20" t="n">
-        <v>35.16317559085985</v>
+        <v>2055.984578196735</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0261948013040817</v>
+        <v>2.185562763901314</v>
       </c>
       <c r="K20" t="n">
         <v>1.25011431627727</v>
@@ -1156,25 +1156,25 @@
         <v>100</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1201146741430924</v>
+        <v>0.149896972200933</v>
       </c>
       <c r="E21" t="n">
-        <v>0.07331226319325701</v>
+        <v>0.1046787260414083</v>
       </c>
       <c r="F21" t="n">
-        <v>2.566420654522169</v>
+        <v>3.314966521968003</v>
       </c>
       <c r="G21" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="H21" t="n">
-        <v>4.356464560582069</v>
+        <v>319.8148679586596</v>
       </c>
       <c r="I21" t="n">
-        <v>36.26921183162201</v>
+        <v>2133.564562798214</v>
       </c>
       <c r="J21" t="n">
-        <v>0.02507788370311485</v>
+        <v>2.084218126635174</v>
       </c>
       <c r="K21" t="n">
         <v>1.290731747181407</v>
@@ -1191,25 +1191,25 @@
         <v>233</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F22" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G22" t="n">
         <v>0.001</v>
       </c>
       <c r="H22" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I22" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J22" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K22" t="n">
         <v>1.221558912811017</v>
@@ -1226,25 +1226,25 @@
         <v>233</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E23" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F23" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G23" t="n">
         <v>0.001</v>
       </c>
       <c r="H23" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I23" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J23" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K23" t="n">
         <v>1.221558912811017</v>
@@ -1261,25 +1261,25 @@
         <v>233</v>
       </c>
       <c r="D24" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F24" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G24" t="n">
         <v>0.001</v>
       </c>
       <c r="H24" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I24" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J24" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K24" t="n">
         <v>1.221558912811017</v>
@@ -1296,25 +1296,25 @@
         <v>233</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F25" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G25" t="n">
         <v>0.001</v>
       </c>
       <c r="H25" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I25" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J25" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K25" t="n">
         <v>1.221558912811017</v>
@@ -1331,25 +1331,25 @@
         <v>233</v>
       </c>
       <c r="D26" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F26" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G26" t="n">
         <v>0.001</v>
       </c>
       <c r="H26" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I26" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J26" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K26" t="n">
         <v>1.221558912811017</v>
@@ -1366,25 +1366,25 @@
         <v>233</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F27" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G27" t="n">
         <v>0.001</v>
       </c>
       <c r="H27" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I27" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J27" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K27" t="n">
         <v>1.221558912811017</v>
@@ -1401,25 +1401,25 @@
         <v>233</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F28" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G28" t="n">
         <v>0.001</v>
       </c>
       <c r="H28" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I28" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J28" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K28" t="n">
         <v>1.221558912811017</v>
@@ -1436,25 +1436,25 @@
         <v>233</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F29" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G29" t="n">
         <v>0.001</v>
       </c>
       <c r="H29" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I29" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J29" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K29" t="n">
         <v>1.221558912811017</v>
@@ -1471,25 +1471,25 @@
         <v>233</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E30" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F30" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G30" t="n">
         <v>0.001</v>
       </c>
       <c r="H30" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I30" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J30" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K30" t="n">
         <v>1.221558912811017</v>
@@ -1506,25 +1506,25 @@
         <v>233</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E31" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F31" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G31" t="n">
         <v>0.001</v>
       </c>
       <c r="H31" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I31" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J31" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K31" t="n">
         <v>1.221558912811017</v>
@@ -1541,25 +1541,25 @@
         <v>233</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E32" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F32" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G32" t="n">
         <v>0.001</v>
       </c>
       <c r="H32" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I32" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J32" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K32" t="n">
         <v>1.221558912811017</v>
@@ -1576,25 +1576,25 @@
         <v>233</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E33" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F33" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G33" t="n">
         <v>0.001</v>
       </c>
       <c r="H33" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I33" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J33" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K33" t="n">
         <v>1.221558912811017</v>
@@ -1611,25 +1611,25 @@
         <v>233</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E34" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F34" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G34" t="n">
         <v>0.001</v>
       </c>
       <c r="H34" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I34" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J34" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K34" t="n">
         <v>1.221558912811017</v>
@@ -1646,25 +1646,25 @@
         <v>233</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E35" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F35" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G35" t="n">
         <v>0.001</v>
       </c>
       <c r="H35" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I35" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J35" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K35" t="n">
         <v>1.221558912811017</v>
@@ -1681,25 +1681,25 @@
         <v>233</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E36" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F36" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G36" t="n">
         <v>0.001</v>
       </c>
       <c r="H36" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I36" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J36" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K36" t="n">
         <v>1.221558912811017</v>
@@ -1716,25 +1716,25 @@
         <v>233</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F37" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G37" t="n">
         <v>0.001</v>
       </c>
       <c r="H37" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I37" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J37" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K37" t="n">
         <v>1.221558912811017</v>
@@ -1751,25 +1751,25 @@
         <v>233</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F38" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G38" t="n">
         <v>0.001</v>
       </c>
       <c r="H38" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I38" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J38" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K38" t="n">
         <v>1.221558912811017</v>
@@ -1786,25 +1786,25 @@
         <v>233</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F39" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G39" t="n">
         <v>0.001</v>
       </c>
       <c r="H39" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I39" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J39" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K39" t="n">
         <v>1.221558912811017</v>
@@ -1821,25 +1821,25 @@
         <v>233</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F40" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G40" t="n">
         <v>0.001</v>
       </c>
       <c r="H40" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I40" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J40" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K40" t="n">
         <v>1.221558912811017</v>
@@ -1856,25 +1856,25 @@
         <v>233</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F41" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G41" t="n">
         <v>0.001</v>
       </c>
       <c r="H41" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I41" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J41" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K41" t="n">
         <v>1.221558912811017</v>
@@ -1891,25 +1891,25 @@
         <v>233</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F42" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G42" t="n">
         <v>0.001</v>
       </c>
       <c r="H42" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I42" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J42" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K42" t="n">
         <v>1.221558912811017</v>
@@ -1926,25 +1926,25 @@
         <v>233</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F43" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G43" t="n">
         <v>0.001</v>
       </c>
       <c r="H43" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I43" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J43" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K43" t="n">
         <v>1.221558912811017</v>
@@ -1961,25 +1961,25 @@
         <v>233</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F44" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G44" t="n">
         <v>0.001</v>
       </c>
       <c r="H44" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I44" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J44" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K44" t="n">
         <v>1.221558912811017</v>
@@ -1996,25 +1996,25 @@
         <v>233</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F45" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G45" t="n">
         <v>0.001</v>
       </c>
       <c r="H45" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I45" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J45" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K45" t="n">
         <v>1.221558912811017</v>
@@ -2031,25 +2031,25 @@
         <v>233</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F46" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G46" t="n">
         <v>0.001</v>
       </c>
       <c r="H46" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I46" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J46" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K46" t="n">
         <v>1.221558912811017</v>
@@ -2066,25 +2066,25 @@
         <v>233</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F47" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G47" t="n">
         <v>0.001</v>
       </c>
       <c r="H47" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I47" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J47" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K47" t="n">
         <v>1.221558912811017</v>
@@ -2101,25 +2101,25 @@
         <v>233</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F48" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G48" t="n">
         <v>0.001</v>
       </c>
       <c r="H48" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I48" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J48" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K48" t="n">
         <v>1.221558912811017</v>
@@ -2136,25 +2136,25 @@
         <v>233</v>
       </c>
       <c r="D49" t="n">
-        <v>0.1811449267518876</v>
+        <v>0.1856235176696466</v>
       </c>
       <c r="E49" t="n">
-        <v>0.1631084713939998</v>
+        <v>0.1676857096888018</v>
       </c>
       <c r="F49" t="n">
-        <v>10.04326643775198</v>
+        <v>10.34817174249318</v>
       </c>
       <c r="G49" t="n">
         <v>0.001</v>
       </c>
       <c r="H49" t="n">
-        <v>19.18414947938523</v>
+        <v>1136.107764509158</v>
       </c>
       <c r="I49" t="n">
-        <v>105.9049779829692</v>
+        <v>6120.49474534301</v>
       </c>
       <c r="J49" t="n">
-        <v>0.07330599712226725</v>
+        <v>4.309345336910132</v>
       </c>
       <c r="K49" t="n">
         <v>1.221558912811017</v>

</xml_diff>